<commit_message>
ventas: fix BUG 2 - 6 partners a Maestra Canales
Maestra Canales: 165 -> 171 filas
- IMPORTADORA Y EXPORTADORA ESTADO LIMITADA -> UnionX B2B
- MineGroup SpA                              -> UnionX B2B
- Teknorpro Chile SpA                        -> UnionX B2B
- Sanchez y Cia.                             -> UnionX B2B
- Shopify Lhotse, Ara Osswald                -> Lhotse web
- Melollevo, Martin Novoa Oficial            -> UnionX web

Resultado: 0 filas mayo sin canal/TN/KAM (antes 16 filas, $5.87 MM)
Parquet: 13,448 filas, $405.83 MM bruta, mayo completo hasta 22-may

S224681 (Melollevo, 8-may) ya estaba cancelado en Odoo state=cancel,
no aparece en el extract (correcto).
</commit_message>
<xml_diff>
--- a/data/planillas/Maestra Canales.xlsx
+++ b/data/planillas/Maestra Canales.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B166"/>
+  <dimension ref="A1:B172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2420,6 +2420,78 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>IMPORTADORA Y EXPORTADORA ESTADO LIMITADA</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>UnionX B2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>MineGroup SpA</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>UnionX B2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Teknorpro Chile SpA</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>UnionX B2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Shopify Lhotse, Ara Osswald</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Lhotse web</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Melollevo, Martin Novoa Oficial</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>UnionX web</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Sanchez y Cia.</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>UnionX B2B</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>